<commit_message>
Modified Order Revenue Data Exploration Files
</commit_message>
<xml_diff>
--- a/Excel_Practice/Data_Exploration/Order_Revenue_Data_Exploration/Order_Revenue_Data_Exploration.xlsx
+++ b/Excel_Practice/Data_Exploration/Order_Revenue_Data_Exploration/Order_Revenue_Data_Exploration.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mani_Entri_DA_Documents\Excel_Practice\Data_Exploration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mani_Entri_DA_Documents\Excel_Practice\Data_Exploration\Order_Revenue_Data_Exploration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED5A8D6-45F0-4F8F-9F06-75FD81D6AF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8905C1CA-E6D9-48B2-8701-DCDD26A47E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="4" xr2:uid="{D6AD5B38-86C7-49E6-9824-04F0B7C3AEA2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D6AD5B38-86C7-49E6-9824-04F0B7C3AEA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Order_Revenue_DB" sheetId="1" r:id="rId1"/>
@@ -1503,16 +1503,6 @@
   <dxfs count="40">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
         <color theme="9" tint="-0.24994659260841701"/>
@@ -1525,6 +1515,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1558,6 +1558,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i/>
         <color theme="9" tint="-0.499984740745262"/>
@@ -1575,13 +1585,10 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <b/>
+        <i val="0"/>
+        <color theme="9" tint="-0.24994659260841701"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1592,13 +1599,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1614,16 +1614,16 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -6601,10 +6601,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="14" priority="33" operator="containsText" text="Low Sales">
+    <cfRule type="containsText" dxfId="14" priority="32" operator="containsText" text="Low Sales">
       <formula>NOT(ISERROR(SEARCH("Low Sales",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="32" operator="containsText" text="Low Sales">
+    <cfRule type="containsText" dxfId="13" priority="33" operator="containsText" text="Low Sales">
       <formula>NOT(ISERROR(SEARCH("Low Sales",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6614,11 +6614,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576">
-    <cfRule type="containsText" dxfId="11" priority="31" operator="containsText" text="TRUE">
+    <cfRule type="containsText" dxfId="11" priority="30" operator="containsText" text="A$K$1">
+      <formula>NOT(ISERROR(SEARCH("A$K$1",K1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="31" operator="containsText" text="TRUE">
       <formula>NOT(ISERROR(SEARCH("TRUE",K1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="30" operator="containsText" text="A$K$1">
-      <formula>NOT(ISERROR(SEARCH("A$K$1",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:M1048576">
@@ -6627,10 +6627,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:L1048576">
-    <cfRule type="containsText" dxfId="8" priority="23" operator="containsText" text="Best Sales">
+    <cfRule type="containsText" dxfId="8" priority="22" operator="containsText" text="Best Sales">
       <formula>NOT(ISERROR(SEARCH("Best Sales",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="22" operator="containsText" text="Best Sales">
+    <cfRule type="containsText" dxfId="7" priority="23" operator="containsText" text="Best Sales">
       <formula>NOT(ISERROR(SEARCH("Best Sales",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6640,24 +6640,24 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:N1048576">
-    <cfRule type="containsText" dxfId="5" priority="25" operator="containsText" text="NOT">
+    <cfRule type="containsText" dxfId="5" priority="24" operator="containsText" text="FALSE">
+      <formula>NOT(ISERROR(SEARCH("FALSE",N1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="25" operator="containsText" text="NOT">
       <formula>NOT(ISERROR(SEARCH("NOT",N1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="24" operator="containsText" text="FALSE">
-      <formula>NOT(ISERROR(SEARCH("FALSE",N1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="26" operator="containsText" text="FALSE">
       <formula>NOT(ISERROR(SEARCH("FALSE",N1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1:U1048576">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="A$K$1">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="TRUE">
+      <formula>NOT(ISERROR(SEARCH("TRUE",O1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="A$K$1">
       <formula>NOT(ISERROR(SEARCH("A$K$1",O1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="TRUE">
-      <formula>NOT(ISERROR(SEARCH("TRUE",O1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="TRUE">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="TRUE">
       <formula>NOT(ISERROR(SEARCH("TRUE",O1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>